<commit_message>
feat(crm): multi-tag system with TagInput component, bulk edit, and tag-based blast targeting
- Add shadcn-style TagInput chip component (components/ui/TagInput.jsx):
  Enter/comma to add, Backspace to remove, dedup case-insensitive,
  suggestions from existing DB tags
- Replace raw comma text inputs with TagInput in add/edit contact modals
- Bulk edit tag section now uses single TagInput field (add/replace/remove)
- Table tag column now renders via Badge component (shadcn convention)
- Broadcast wizard: target by group or multi-tag with OR/AND match mode,
  live recipient estimate, target_type/target_tags persisted to wa_campaigns
- Fix SPA staleness: refreshContacts now re-fetches on every tab change;
  edit-contact handler now also triggers global contacts refresh
- Backend: bulk-update & bulk-delete endpoints, tag column expansion
  migration (VARCHAR 500), Excel template now includes tag column
</commit_message>
<xml_diff>
--- a/public/template-kontak-blast.xlsx
+++ b/public/template-kontak-blast.xlsx
@@ -551,16 +551,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -586,22 +587,27 @@
           <t>group</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>tag</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>kota</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>voucher</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>nominal</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>link</t>
         </is>
@@ -623,22 +629,27 @@
           <t>Pelanggan VIP</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>VIP, Jakarta, Prioritas</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>Jakarta</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>PROMO100K</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>100.000</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>https://srvx.id/v/budi</t>
         </is>
@@ -660,22 +671,27 @@
           <t>Reseller Reguler</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Reseller, Surabaya</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>Surabaya</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>DISC25</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>50.000</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>https://srvx.id/v/siti</t>
         </is>
@@ -689,7 +705,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>+6281987654321</t>
+          <t>+6281234564321</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -697,22 +713,27 @@
           <t>Lead Prospek</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Hot Lead, Promo</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>Bandung</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>NEWUSER</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>25.000</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>https://srvx.id/v/ahmad</t>
         </is>
@@ -734,22 +755,27 @@
           <t>Pelanggan VIP</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>VIP, Medan</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>Medan</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>VIP50</t>
         </is>
       </c>
-      <c r="F6" s="11" t="inlineStr">
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>150.000</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>https://srvx.id/v/dewi</t>
         </is>
@@ -771,22 +797,27 @@
           <t>Reseller Reguler</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Reseller, Jogja</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Yogyakarta</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>CASHBACK</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>75.000</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>https://srvx.id/v/rian</t>
         </is>
@@ -794,7 +825,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -806,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -892,32 +923,49 @@
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>Variabel Kustom</t>
+          <t>tag</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Semua kolom tambahan di samping kanan kolom group (misal: kota, voucher, tagihan, dll) otomatis disimpan sebagai Variabel Kustom Kontak.</t>
+          <t>Tag atau label kontak (Opsional). Bisa multi-tag dipisahkan dengan koma.</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Kolom baru: tagihan, tenor, dsb</t>
+          <t>VIP, Jakarta, Member</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
+          <t>Variabel Kustom</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Semua kolom tambahan di samping kanan kolom tag (misal: kota, voucher, tagihan, dll) otomatis disimpan sebagai Variabel Kustom Kontak.</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Kolom baru: tagihan, tenor, dsb</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
           <t>Cara Panggil</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Di template pesan WA Blast, panggil menggunakan format kurung kurawal ganda.</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>Halo {{name}}, voucher Anda {{voucher}} di {{kota}}</t>
         </is>

</xml_diff>